<commit_message>
Update resources and Pages configuration
</commit_message>
<xml_diff>
--- a/AI_Bridge_자료실_링크.xlsx
+++ b/AI_Bridge_자료실_링크.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료실" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'자료실'!$A$1:$F$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'자료실'!$A$1:$F$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1481,17 +1481,17 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>RunwayML</t>
+          <t>lobe</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>https://runwayml.com</t>
+          <t>https://www.lobe.ai</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>코드 없이 사용하는 AI 영상·이미지 생성 도구. 배경 제거, 모션 추적, AI 영상 편집 지원</t>
+          <t>Microsoft의 코드 없는 이미지 분류 AI 학습 도구. 사진만 모으면 분류 모델 생성 가능</t>
         </is>
       </c>
     </row>
@@ -1511,17 +1511,17 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>lobe</t>
+          <t>Brightics AI (삼성)</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>https://www.lobe.ai</t>
+          <t>https://www.brightics.ai</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Microsoft의 코드 없는 이미지 분류 AI 학습 도구. 사진만 모으면 분류 모델 생성 가능</t>
+          <t>삼성SDS의 노코드 AI 분석 플랫폼. 제조·유통·금융 데이터 분석에 특화된 기업용 도구</t>
         </is>
       </c>
     </row>
@@ -1536,22 +1536,22 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>5. No Code AI 도구</t>
+          <t>6. 제작·디자인 도구</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Brightics AI (삼성)</t>
+          <t>Gamma</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>https://www.brightics.ai</t>
+          <t>https://gamma.app</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>삼성SDS의 노코드 AI 분석 플랫폼. 제조·유통·금융 데이터 분석에 특화된 기업용 도구</t>
+          <t>AI로 프레젠테이션·문서·웹페이지를 빠르게 제작. 텍스트 입력만으로 슬라이드 자동 생성</t>
         </is>
       </c>
     </row>
@@ -1571,17 +1571,17 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Gamma</t>
+          <t>Canva</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>https://gamma.app</t>
+          <t>https://www.canva.com</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>AI로 프레젠테이션·문서·웹페이지를 빠르게 제작. 텍스트 입력만으로 슬라이드 자동 생성</t>
+          <t>드래그앤드롭 방식의 범용 디자인 도구. Magic Write 등 AI 기능 내장</t>
         </is>
       </c>
     </row>
@@ -1601,17 +1601,17 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Canva</t>
+          <t>미리캔버스</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>https://www.canva.com</t>
+          <t>https://www.miricanvas.com</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>드래그앤드롭 방식의 범용 디자인 도구. Magic Write 등 AI 기능 내장</t>
+          <t>한국어 특화 무료 디자인 도구. 교육용 템플릿 다수 제공</t>
         </is>
       </c>
     </row>
@@ -1631,17 +1631,17 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>미리캔버스</t>
+          <t>망고보드</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>https://www.miricanvas.com</t>
+          <t>https://www.mangoboard.net</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>한국어 특화 무료 디자인 도구. 교육용 템플릿 다수 제공</t>
+          <t>한국형 인포그래픽·카드뉴스·PPT 제작 도구. 교육 현장에서 많이 활용</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1661,17 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>망고보드</t>
+          <t>투닝</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>https://www.mangoboard.net</t>
+          <t>https://tooning.io</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>한국형 인포그래픽·카드뉴스·PPT 제작 도구. 교육 현장에서 많이 활용</t>
+          <t>AI 기반 웹툰·만화 제작 도구. 캐릭터와 배경을 자동 생성해 학습 만화 제작 가능</t>
         </is>
       </c>
     </row>
@@ -1691,17 +1691,17 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>투닝</t>
+          <t>Figma</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>https://tooning.io</t>
+          <t>https://www.figma.com</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>AI 기반 웹툰·만화 제작 도구. 캐릭터와 배경을 자동 생성해 학습 만화 제작 가능</t>
+          <t>UI/UX 디자인 협업 도구. AI 플러그인 다수 지원. 교육용 무료 플랜 제공</t>
         </is>
       </c>
     </row>
@@ -1711,27 +1711,27 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>AI 기초 이해</t>
+          <t>수업 지원</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>6. 제작·디자인 도구</t>
+          <t>1. 한글·문해 수업 자료</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Figma</t>
+          <t>온한글</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>https://www.figma.com</t>
+          <t>https://onhan.cne.go.kr/</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>UI/UX 디자인 협업 도구. AI 플러그인 다수 지원. 교육용 무료 플랜 제공</t>
+          <t>충청남도교육청 한글 해득 진단·보정 시스템. 미해득 학생 보정 자료와 성장 기록 지원</t>
         </is>
       </c>
     </row>
@@ -1746,22 +1746,22 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>1. 한글·문해 수업 자료</t>
+          <t>2. 창작·스몰 도구</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>온한글</t>
+          <t>Chrome Music Lab</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>https://onhan.cne.go.kr/</t>
+          <t>https://musiclab.chromeexperiments.com/</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>충청남도교육청 한글 해득 진단·보정 시스템. 미해득 학생 보정 자료와 성장 기록 지원</t>
+          <t>리듬, 멜로디, 소리의 파형을 놀이처럼 탐색하는 구글의 웹 기반 음악 실험실</t>
         </is>
       </c>
     </row>
@@ -1781,17 +1781,17 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Chrome Music Lab</t>
+          <t>AutoDraw</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>https://musiclab.chromeexperiments.com/</t>
+          <t>https://www.autodraw.com/</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>리듬, 멜로디, 소리의 파형을 놀이처럼 탐색하는 구글의 웹 기반 음악 실험실</t>
+          <t>간단한 스케치를 AI가 그림 아이콘으로 추천해 주는 구글 크리에이티브 랩의 드로잉 도구</t>
         </is>
       </c>
     </row>
@@ -1806,22 +1806,22 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>2. 창작·스몰 도구</t>
+          <t>3. 프로그래밍 수업 도구</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>AutoDraw</t>
+          <t>Delightex Edu</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>https://www.autodraw.com/</t>
+          <t>https://www.delightex.com/edu</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>간단한 스케치를 AI가 그림 아이콘으로 추천해 주는 구글 크리에이티브 랩의 드로잉 도구</t>
+          <t>3D 공간, VR·AR 콘텐츠를 만들고 블록 코딩과 스크립트로 상호작용을 구현하는 교육용 제작 도구</t>
         </is>
       </c>
     </row>
@@ -1841,17 +1841,17 @@
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Delightex Edu</t>
+          <t>엔트리</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>https://www.delightex.com/edu</t>
+          <t>https://playentry.org/ko/</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>3D 공간, VR·AR 콘텐츠를 만들고 블록 코딩과 스크립트로 상호작용을 구현하는 교육용 제작 도구</t>
+          <t>네이버 커넥트재단에서 운영하는 비영리 블록 코딩 교육 플랫폼</t>
         </is>
       </c>
     </row>
@@ -1871,17 +1871,17 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>엔트리</t>
+          <t>스크래치</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>https://playentry.org/ko/</t>
+          <t>https://scratch.mit.edu/</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>네이버 커넥트재단에서 운영하는 비영리 블록 코딩 교육 플랫폼</t>
+          <t>스토리, 게임, 애니메이션을 만들며 프로그래밍 기초를 배우는 블록 기반 창작 플랫폼</t>
         </is>
       </c>
     </row>
@@ -1896,22 +1896,22 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>3. 프로그래밍 수업 도구</t>
+          <t>4. 시뮬레이션 수업 도구</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>스크래치</t>
+          <t>자바실험실</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>https://scratch.mit.edu/</t>
+          <t>https://javalab.org/ko/</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>스토리, 게임, 애니메이션을 만들며 프로그래밍 기초를 배우는 블록 기반 창작 플랫폼</t>
+          <t>과학·수학 개념을 웹 시뮬레이션으로 탐구할 수 있는 한국어 실험 자료 사이트</t>
         </is>
       </c>
     </row>
@@ -1931,17 +1931,17 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>자바실험실</t>
+          <t>지오지브라</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>https://javalab.org/ko/</t>
+          <t>https://www.geogebra.org/?lang=ko</t>
         </is>
       </c>
       <c r="F49" s="3" t="inlineStr">
         <is>
-          <t>과학·수학 개념을 웹 시뮬레이션으로 탐구할 수 있는 한국어 실험 자료 사이트</t>
+          <t>함수, 기하, 통계, 3D 그래프 등을 조작하며 탐구하는 수학 시뮬레이션 플랫폼</t>
         </is>
       </c>
     </row>
@@ -1961,17 +1961,17 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>지오지브라</t>
+          <t>알지오매스</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>https://www.geogebra.org/?lang=ko</t>
+          <t>https://www.algeomath.kr/</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
         <is>
-          <t>함수, 기하, 통계, 3D 그래프 등을 조작하며 탐구하는 수학 시뮬레이션 플랫폼</t>
+          <t>수학 개념을 그래프와 기하 모델로 시각화해 수업에 활용할 수 있는 국내 수학 탐구 도구</t>
         </is>
       </c>
     </row>
@@ -1991,17 +1991,17 @@
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>알지오매스</t>
+          <t>VlabON</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>https://www.algeomath.kr/</t>
+          <t>https://www.vlabon.re.kr/</t>
         </is>
       </c>
       <c r="F51" s="3" t="inlineStr">
         <is>
-          <t>수학 개념을 그래프와 기하 모델로 시각화해 수업에 활용할 수 있는 국내 수학 탐구 도구</t>
+          <t>가상 실험과 과학 탐구 활동을 지원하는 온라인 과학 실험 플랫폼</t>
         </is>
       </c>
     </row>
@@ -2016,22 +2016,22 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>4. 시뮬레이션 수업 도구</t>
+          <t>5. AI 교육 포털</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>VlabON</t>
+          <t>에듀넷 AI·SW 교육</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>https://www.vlabon.re.kr/</t>
+          <t>https://ai.edunet.net</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>가상 실험과 과학 탐구 활동을 지원하는 온라인 과학 실험 플랫폼</t>
+          <t>교육부 공식 AI·SW 교육 포털. 교사·학생용 자료, 연수, 수업 지원 통합 제공</t>
         </is>
       </c>
     </row>
@@ -2051,17 +2051,17 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>에듀넷 AI·SW 교육</t>
+          <t>에듀넷 티-클리어 AI 교수학습자료</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>https://ai.edunet.net</t>
+          <t>https://ai.edunet.net/aiTchLrngData/list/408</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>교육부 공식 AI·SW 교육 포털. 교사·학생용 자료, 연수, 수업 지원 통합 제공</t>
+          <t>에듀넷의 AI 교수·학습 자료 목록. 수업에서 바로 활용 가능한 자료 모음</t>
         </is>
       </c>
     </row>
@@ -2081,17 +2081,17 @@
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>에듀넷 티-클리어 AI 교수학습자료</t>
+          <t>에듀넷 AI·SW 연구·기타자료</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>https://ai.edunet.net/aiTchLrngData/list/408</t>
+          <t>https://ai.edunet.net/aiStdyEtcData/list/411</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
         <is>
-          <t>에듀넷의 AI 교수·학습 자료 목록. 수업에서 바로 활용 가능한 자료 모음</t>
+          <t>AI·SW 교육 관련 연구 보고서 및 기타 참고 자료</t>
         </is>
       </c>
     </row>
@@ -2111,17 +2111,17 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>에듀넷 AI·SW 연구·기타자료</t>
+          <t>한국과학창의재단 SAI</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>https://ai.edunet.net/aiStdyEtcData/list/411</t>
+          <t>https://www.kosac.re.kr/menus/1124/contents/1124</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>AI·SW 교육 관련 연구 보고서 및 기타 참고 자료</t>
+          <t>한국과학창의재단의 학교 AI 교육(SAI) 사업 안내 및 자료 제공 페이지</t>
         </is>
       </c>
     </row>
@@ -2141,17 +2141,17 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>한국과학창의재단 SAI</t>
+          <t>SAI 교육콘텐츠</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>https://www.kosac.re.kr/menus/1124/contents/1124</t>
+          <t>https://sai.software.kr</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>한국과학창의재단의 학교 AI 교육(SAI) 사업 안내 및 자료 제공 페이지</t>
+          <t>학교 AI 교육을 위한 교육콘텐츠·수업 자료 포털</t>
         </is>
       </c>
     </row>
@@ -2171,17 +2171,17 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>SAI 교육콘텐츠</t>
+          <t>AI·디지털 교육자료 수업지원센터</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>https://sai.software.kr</t>
+          <t>https://www.ai-dt.net</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>학교 AI 교육을 위한 교육콘텐츠·수업 자료 포털</t>
+          <t>교사가 AI·디지털 교육자료를 찾고 수업에 바로 적용할 수 있는 지원 센터</t>
         </is>
       </c>
     </row>
@@ -2201,17 +2201,17 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>AI·디지털 교육자료 수업지원센터</t>
+          <t>AI·디지털 교육자료(aidtbook)</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>https://www.ai-dt.net</t>
+          <t>https://www.aidtbook.kr/index.do</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>교사가 AI·디지털 교육자료를 찾고 수업에 바로 적용할 수 있는 지원 센터</t>
+          <t>AI 디지털 교과서 관련 교육자료 통합 제공 포털</t>
         </is>
       </c>
     </row>
@@ -2231,17 +2231,17 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>AI·디지털 교육자료(aidtbook)</t>
+          <t>미래엔 AI·디지털 교육자료</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>https://www.aidtbook.kr/index.do</t>
+          <t>https://aidt.m-teacher.co.kr</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>AI 디지털 교과서 관련 교육자료 통합 제공 포털</t>
+          <t>출판사 미래엔에서 제공하는 AI·디지털 교육자료 및 교사 지원 자료</t>
         </is>
       </c>
     </row>
@@ -2261,17 +2261,17 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>미래엔 AI·디지털 교육자료</t>
+          <t>아이스크림 AI 디지털 교육자료</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>https://aidt.m-teacher.co.kr</t>
+          <t>https://aidt.i-scream.co.kr</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>출판사 미래엔에서 제공하는 AI·디지털 교육자료 및 교사 지원 자료</t>
+          <t>아이스크림미디어의 AI 디지털 교육자료 플랫폼. 초등 특화 콘텐츠 다수</t>
         </is>
       </c>
     </row>
@@ -2291,17 +2291,17 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>아이스크림 AI 디지털 교육자료</t>
+          <t>빛고을 아이(AI) — 광주 AI 교육 프로그램</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>https://aidt.i-scream.co.kr</t>
+          <t>https://sw.gen.go.kr/bbs/board.php?bo_table=data&amp;wr_id=15</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>아이스크림미디어의 AI 디지털 교육자료 플랫폼. 초등 특화 콘텐츠 다수</t>
+          <t>광주 AI 교육센터가 2024년에 공개한 초등용 AI 교육 프로그램 교재</t>
         </is>
       </c>
     </row>
@@ -2321,17 +2321,17 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>빛고을 아이(AI) — 광주 AI 교육 프로그램</t>
+          <t>울산교육청 우리아이</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>https://sw.gen.go.kr/bbs/board.php?bo_table=data&amp;wr_id=15</t>
+          <t>https://wooriai.use.go.kr/</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>광주 AI 교육센터가 2024년에 공개한 초등용 AI 교육 프로그램 교재</t>
+          <t>울산광역시교육청에서 운영하는 학생용 AI 챗봇 서비스</t>
         </is>
       </c>
     </row>
@@ -2351,17 +2351,17 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>울산교육청 우리아이</t>
+          <t>초·중등 AI 수학 융합교육 교수학습자료</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>https://wooriai.use.go.kr/</t>
+          <t>https://sw.gen.go.kr/bbs/board.php?bo_table=data&amp;wr_id=64</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>울산광역시교육청에서 운영하는 학생용 AI 챗봇 서비스</t>
+          <t>광주 SW 교육지원센터가 2024년에 발간한 초·중등 인공지능-수학 융합 수업 자료</t>
         </is>
       </c>
     </row>
@@ -2381,17 +2381,17 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>초·중등 AI 수학 융합교육 교수학습자료</t>
+          <t>초등인공지능교육.COM</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>https://sw.gen.go.kr/bbs/board.php?bo_table=data&amp;wr_id=64</t>
+          <t>https://www.xn--ob0bug89lftci99a2oa25k5pi.com/</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>광주 SW 교육지원센터가 2024년에 발간한 초·중등 인공지능-수학 융합 수업 자료</t>
+          <t>초등 교사가 직접 운영하는 인공지능 수업 자료 모음 사이트</t>
         </is>
       </c>
     </row>
@@ -2411,17 +2411,17 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>초등인공지능교육.COM</t>
+          <t>VIVASAM 초등 인공지능 자료</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>https://www.xn--ob0bug89lftci99a2oa25k5pi.com/</t>
+          <t>https://e.vivasam.com/creative/edu/sw/cia/list</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>초등 교사가 직접 운영하는 인공지능 수업 자료 모음 사이트</t>
+          <t>비상교육 비바샘에서 제공하는 초등 인공지능·창의 수업 자료 모음</t>
         </is>
       </c>
     </row>
@@ -2441,17 +2441,17 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>VIVASAM 초등 인공지능 자료</t>
+          <t>초등 인공지능 교육 모듈형 39강좌</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>https://e.vivasam.com/creative/edu/sw/cia/list</t>
+          <t>https://sites.google.com/ptsaebit.es.kr/metaverse/%EC%B4%88%EB%93%B1swai-%EC%BD%98%ED%85%90%EC%B8%A0-%EB%AA%A8%EC%9D%8C/%EC%B4%88%EB%93%B1-%EC%9D%B8%EA%B3%B5%EC%A7%80%EB%8A%A5-%EA%B5%90%EC%9C%A1%EB%AA%A8%EB%93%88%ED%98%95-39%EA%B0%95%EC%A2%8C</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>비상교육 비바샘에서 제공하는 초등 인공지능·창의 수업 자료 모음</t>
+          <t>초등 단계의 인공지능 교육을 모듈형 39강좌로 구성한 교사용 콘텐츠 모음</t>
         </is>
       </c>
     </row>
@@ -2471,17 +2471,17 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>초등 인공지능 교육 모듈형 39강좌</t>
+          <t>소프트웨어야 놀자</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>https://sites.google.com/ptsaebit.es.kr/metaverse/%EC%B4%88%EB%93%B1swai-%EC%BD%98%ED%85%90%EC%B8%A0-%EB%AA%A8%EC%9D%8C/%EC%B4%88%EB%93%B1-%EC%9D%B8%EA%B3%B5%EC%A7%80%EB%8A%A5-%EA%B5%90%EC%9C%A1%EB%AA%A8%EB%93%88%ED%98%95-39%EA%B0%95%EC%A2%8C</t>
+          <t>https://www.playsw.or.kr/main</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>초등 단계의 인공지능 교육을 모듈형 39강좌로 구성한 교사용 콘텐츠 모음</t>
+          <t>네이버커넥트재단이 운영하는 SW·AI 교육 콘텐츠 플랫폼</t>
         </is>
       </c>
     </row>
@@ -2501,17 +2501,17 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>소프트웨어야 놀자</t>
+          <t>씨마스 AI 디지털 교육자료</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>https://www.playsw.or.kr/main</t>
+          <t>https://viewer.cmass.kr/html/aidt/aidt_e/view_aidt_e.html</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>네이버커넥트재단이 운영하는 SW·AI 교육 콘텐츠 플랫폼</t>
+          <t>씨마스가 제공하는 AI 디지털 교과서 미리보기·교육자료</t>
         </is>
       </c>
     </row>
@@ -2531,17 +2531,17 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>씨마스 AI 디지털 교육자료</t>
+          <t>천재교육 AI 디지털 교육자료 지원센터</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>https://viewer.cmass.kr/html/aidt/aidt_e/view_aidt_e.html</t>
+          <t>https://support.aitextbook.co.kr/</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>씨마스가 제공하는 AI 디지털 교과서 미리보기·교육자료</t>
+          <t>천재교육의 AI 디지털 교과서 활용 안내 및 교사 지원 자료</t>
         </is>
       </c>
     </row>
@@ -2561,17 +2561,17 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>천재교육 AI 디지털 교육자료 지원센터</t>
+          <t>MyAI Edu</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>https://support.aitextbook.co.kr/</t>
+          <t>https://myai.kr/</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>천재교육의 AI 디지털 교과서 활용 안내 및 교사 지원 자료</t>
+          <t>교사·학생을 위한 인공지능 교육 통합 콘텐츠 사이트</t>
         </is>
       </c>
     </row>
@@ -2591,17 +2591,17 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>MyAI Edu</t>
+          <t>인공지능 교육자료 사이트 모음(노션)</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>https://myai.kr/</t>
+          <t>https://ai4edu.notion.site/AI-92b8c8eca0294fc7a9a2538bca205bdf</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>교사·학생을 위한 인공지능 교육 통합 콘텐츠 사이트</t>
+          <t>이준기·김귀훈 선생님이 정리한 국내외 AI 교육자료 링크 모음 노션 페이지</t>
         </is>
       </c>
     </row>
@@ -2611,27 +2611,27 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>수업 지원</t>
+          <t>행정 업무</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>5. AI 교육 포털</t>
+          <t>학교업무 도움자료</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>인공지능 교육자료 사이트 모음(노션)</t>
+          <t>경상남도교육청 학교업무 도움자료</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>https://ai4edu.notion.site/AI-92b8c8eca0294fc7a9a2538bca205bdf</t>
+          <t>https://hryoon0.github.io/helppage/</t>
         </is>
       </c>
       <c r="F72" s="3" t="inlineStr">
         <is>
-          <t>이준기·김귀훈 선생님이 정리한 국내외 AI 교육자료 링크 모음 노션 페이지</t>
+          <t>경상남도교육청 학교업무 도움자료 사이트. 초등학교 업무 참고 자료를 확인할 수 있습니다.</t>
         </is>
       </c>
     </row>
@@ -2641,27 +2641,27 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>행정 업무</t>
+          <t>연구·연수·기타</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>학교업무 도움자료</t>
+          <t>1. 연구</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>경상남도교육청 학교업무 도움자료</t>
+          <t>AIEDAP AI융합교육 학술자료</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>https://hryoon0.github.io/helppage/</t>
+          <t>https://aiedap.or.kr/ai융합수업-지원/ai융합교육-학술자료/</t>
         </is>
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>경상남도교육청 학교업무 도움자료 사이트. 초등학교 업무 참고 자료를 확인할 수 있습니다.</t>
+          <t>AI 융합교육 관련 학술 논문·연구 보고서를 모아둔 AIEDAP 공식 페이지</t>
         </is>
       </c>
     </row>
@@ -2681,17 +2681,17 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>AIEDAP AI융합교육 학술자료</t>
+          <t>한국과학창의재단 연구보고서</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>https://aiedap.or.kr/ai융합수업-지원/ai융합교육-학술자료/</t>
+          <t>https://www.kosac.re.kr/menus/244/boards/457/posts</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>AI 융합교육 관련 학술 논문·연구 보고서를 모아둔 AIEDAP 공식 페이지</t>
+          <t>한국과학창의재단이 발간한 과학·수학·정보·융합 교육 분야 연구보고서 모음</t>
         </is>
       </c>
     </row>
@@ -2711,17 +2711,17 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>한국과학창의재단 연구보고서</t>
+          <t>한국인공지능교육학회</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>https://www.kosac.re.kr/menus/244/boards/457/posts</t>
+          <t>http://aied.or.kr/</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>한국과학창의재단이 발간한 과학·수학·정보·융합 교육 분야 연구보고서 모음</t>
+          <t>인공지능 교육 연구를 전문으로 하는 학술 단체. 학술지·학술대회 정보 제공</t>
         </is>
       </c>
     </row>
@@ -2736,22 +2736,22 @@
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>1. 연구</t>
+          <t>2. 연수</t>
         </is>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>한국인공지능교육학회</t>
+          <t>KERIS 종합교육연수원 연수 자료집</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>http://aied.or.kr/</t>
+          <t>https://www.cet.keris.or.kr/usr/reference/selectTrainingListPageVw.do?menuNo=23100</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>인공지능 교육 연구를 전문으로 하는 학술 단체. 학술지·학술대회 정보 제공</t>
+          <t>KERIS 종합교육연수원에서 제공하는 교원 연수 자료집 모음</t>
         </is>
       </c>
     </row>
@@ -2766,22 +2766,22 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>2. 연수</t>
+          <t>3. 기타</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>KERIS 종합교육연수원 연수 자료집</t>
+          <t>교과 학습발달상황 작성 GPT</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>https://www.cet.keris.or.kr/usr/reference/selectTrainingListPageVw.do?menuNo=23100</t>
+          <t>https://chatgpt.com/g/g-6753f78947708191b221bbf659619dfd-seongcwigijun-giban-gyogwahagseubbaldalsanghwang-saengseong-caesbos-jeongwamog</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>KERIS 종합교육연수원에서 제공하는 교원 연수 자료집 모음</t>
+          <t>ChatGPT 커스텀 GPT. 학생의 학습 활동·성과를 입력하면 교과 학습발달상황을 자동으로 생성</t>
         </is>
       </c>
     </row>
@@ -2801,17 +2801,17 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>교과 학습발달상황 작성 GPT</t>
+          <t>교육 아이디어 도우미 GPT</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>https://chatgpt.com/g/g-6753f78947708191b221bbf659619dfd-seongcwigijun-giban-gyogwahagseubbaldalsanghwang-saengseong-caesbos-jeongwamog</t>
+          <t>https://chatgpt.com/g/g-677cab3951bc8191adf633bd9e6b9fcb-gyoyug-aidieo-doumi</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>ChatGPT 커스텀 GPT. 학생의 학습 활동·성과를 입력하면 교과 학습발달상황을 자동으로 생성</t>
+          <t>ChatGPT 커스텀 GPT. 수업 주제·상황을 입력하면 교육 활동 아이디어를 제안해 주는 도우미</t>
         </is>
       </c>
     </row>
@@ -2831,52 +2831,22 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>교육 아이디어 도우미 GPT</t>
+          <t>교육·다큐멘터리·어학·어린이 유튜브 영상 보기 GPT</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>https://chatgpt.com/g/g-677cab3951bc8191adf633bd9e6b9fcb-gyoyug-aidieo-doumi</t>
+          <t>https://chatgpt.com/g/g-f7aSrkPEP-gyoyug-dakyumenteori-eohag-eorini-yutyubeu-yeongsang-bogi-education</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>ChatGPT 커스텀 GPT. 수업 주제·상황을 입력하면 교육 활동 아이디어를 제안해 주는 도우미</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>연구·연수·기타</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>3. 기타</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>교육·다큐멘터리·어학·어린이 유튜브 영상 보기 GPT</t>
-        </is>
-      </c>
-      <c r="E80" s="4" t="inlineStr">
-        <is>
-          <t>https://chatgpt.com/g/g-f7aSrkPEP-gyoyug-dakyumenteori-eohag-eorini-yutyubeu-yeongsang-bogi-education</t>
-        </is>
-      </c>
-      <c r="F80" s="3" t="inlineStr">
-        <is>
           <t>ChatGPT 커스텀 GPT. 교육·다큐멘터리·어학·어린이 분야의 유튜브 영상을 추천하고 함께 시청·정리할 수 있는 도우미</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F80"/>
+  <autoFilter ref="A1:F79"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -2956,7 +2926,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E77" r:id="rId76"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E78" r:id="rId77"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E79" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E80" r:id="rId79"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>